<commit_message>
Pricing v2 (May 2026 stack): MARKETING_PLAN + AI COGS sensitivity
- Launch £89 setup + £168/yr annual (or £204/yr monthly)
- Growth £468/yr
- Blended ARPU lifted £180 → £200/yr; TAM today ~£62M/yr
- AI COGS + kept-sandbox-as-dev-env (£1.50/mo) folded into margin model
- Year-1 net per customer reflowed across Launch / Growth scenarios

AI_COGS_SENSITIVITY.xlsx: sensitivity table + named cells updated to match.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/proposals/hatchik/AI_COGS_SENSITIVITY.xlsx
+++ b/proposals/hatchik/AI_COGS_SENSITIVITY.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -14,14 +14,17 @@
     <sheet name="Cohort projection" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="false" name="affiliate_per_customer" vbProcedure="false">Inputs!$B$48</definedName>
     <definedName function="false" hidden="false" name="allow_growth" vbProcedure="false">Inputs!$B$19</definedName>
     <definedName function="false" hidden="false" name="allow_launch" vbProcedure="false">Inputs!$B$18</definedName>
+    <definedName function="false" hidden="false" name="annual_rate" vbProcedure="false">Inputs!$B$47</definedName>
     <definedName function="false" hidden="false" name="byo_pct" vbProcedure="false">Inputs!$B$26</definedName>
     <definedName function="false" hidden="false" name="cohort_launch_pct" vbProcedure="false">Inputs!$B$41</definedName>
     <definedName function="false" hidden="false" name="cohort_total" vbProcedure="false">Inputs!$B$40</definedName>
     <definedName function="false" hidden="false" name="cost_blended" vbProcedure="false">Inputs!$B$44</definedName>
     <definedName function="false" hidden="false" name="cost_cheap" vbProcedure="false">Inputs!$B$22</definedName>
     <definedName function="false" hidden="false" name="cost_expensive" vbProcedure="false">Inputs!$B$23</definedName>
+    <definedName function="false" hidden="false" name="float_per_annual" vbProcedure="false">Inputs!$B$49</definedName>
     <definedName function="false" hidden="false" name="infra_cost" vbProcedure="false">Inputs!$B$35</definedName>
     <definedName function="false" hidden="false" name="kept_sandbox_cost" vbProcedure="false">Inputs!$B$38</definedName>
     <definedName function="false" hidden="false" name="margin_growth_mid" vbProcedure="false">'Per-customer margin'!$F$21</definedName>
@@ -53,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="121">
   <si>
     <t xml:space="preserve">Hatchik — AI COGS Sensitivity</t>
   </si>
@@ -63,11 +66,12 @@
   <si>
     <t xml:space="preserve">HOW TO USE THIS
 1. All yellow cells on this sheet are inputs — change them to model your own assumptions.
-2. Per-customer margin (Sheet 2) recomputes automatically. Three scenarios are pre-wired: Pessimistic, Mid-range (uses your inputs as-is), Optimistic.
-3. Sensitivity tables (Sheet 3) show how Launch + Growth margins move as BYO% and utilisation vary, plus a break-even grid.
-4. Cohort projection (Sheet 4) scales the mid-range to 1000 customers at 80/20 Launch/Growth mix.
-5. Tunable strategic lever: the OVERAGE MARKUP cell (B30) controls how much we charge over provider cost for tokens past the included allowance.
-6. NEW (option A — kept sandbox as dev env): the kept_sandbox_cost input (B38) subtracts £1.50/mo from both Launch and Growth margins, modelling the cost of keeping the customer's sandbox alive as a dev environment after they upgrade. Set this cell to 0 if the founder later decides to make the kept-alive sandbox opt-in or to bill it as a separate line item.</t>
+2. Per-customer margin (Sheet 2) recomputes automatically. Three scenarios: Pessimistic (BYO 0%, util 100%, no overage), Mid (= your inputs as-is), Optimistic (BYO 80%, util 20%, some overage).
+3. OVERAGE MODEL — pass-through. Customer pays provider_cost × (1 + overage_markup). Default markup = 60% (bakes in Paddle pass-through + 40% Hatchik margin). Realised as PAYG real-time top-up packs (£5 min) — no monthly settlement = no credit risk.
+4. SUB PRICING — dual structure. Annual £14/mo equiv (£168/yr prepaid). Monthly £17/mo (annual + 15% premium). Blend at the take-rate input drives the model.
+5. KEPT-SANDBOX cost £0.30/mo — drop Studio container, CAX31 host, memory overcommit, 2h idle-suspend. Studio is now a Launch+ feature only.
+6. INFRA cost-to-serve £2.46/mo — shared multi-tenant Launch host on CAX41 (25 tenants/box) + 3 mailboxes. Dedicated VPS reserved for Growth tier.
+7. AFFILIATE revenue £0.10/mo amortised — Cursor/Anthropic/Lovable/Bolt/Windsurf referrals at 5% take rate.</t>
   </si>
   <si>
     <t xml:space="preserve">PRICING</t>
@@ -76,6 +80,9 @@
     <t xml:space="preserve">Launch monthly fee (£)</t>
   </si>
   <si>
+    <t xml:space="preserve">BLENDED. £14/mo equiv on annual (£168/yr prepaid) + £17/mo monthly. Default mix: 40% annual / 60% monthly = (0.4×14 + 0.6×17) = £15.80 weighted-avg revenue per Launch customer. Deck/marketing reference the dual prices; the model uses the blend.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Growth monthly fee (£)</t>
   </si>
   <si>
@@ -139,7 +146,7 @@
     <t xml:space="preserve">Overage markup % (over provider cost)</t>
   </si>
   <si>
-    <t xml:space="preserve">30% default — tunable lever</t>
+    <t xml:space="preserve">60% — bakes in Paddle pass-through (£0.40 fixed + 5%) on top of 40% Hatchik net margin. Overage = real-time PAYG top-up packs (£5 min) — no monthly settlement, no credit risk.</t>
   </si>
   <si>
     <t xml:space="preserve">Avg overage £ provider-cost per Launch non-BYO/mo</t>
@@ -160,7 +167,7 @@
     <t xml:space="preserve">Infra cost-to-serve (£/mo per customer)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hetzner VPS + backups + mail + monitoring</t>
+    <t xml:space="preserve">Shared multi-tenant Launch host on CAX41 (25 tenants × £0.86/mo compute) + 3 mailboxes (£1.50) + backups (£0.20) + monitoring (£0.50). Dedicated VPS reserved for Growth tier (auto-triggered at customer 15th end-user signup).</t>
   </si>
   <si>
     <t xml:space="preserve">Paddle fees — variable %</t>
@@ -178,7 +185,7 @@
     <t xml:space="preserve">Kept-sandbox cost (£/mo per promoted customer)</t>
   </si>
   <si>
-    <t xml:space="preserve">CAX21 host €8/mo ÷ ~5 sandboxes; set to 0 to model opt-in/separate-billing</t>
+    <t xml:space="preserve">CAX31 ÷ ~45 sandboxes (density: drop Studio + memory overcommit + 2h idle-suspend; was £0.60 at 20-sandbox baseline, was £1.50 at original 7-sandbox CAX21 baseline). Studio now Launch+ only.</t>
   </si>
   <si>
     <t xml:space="preserve">COHORT MIX (Sheet 4)</t>
@@ -205,6 +212,27 @@
     <t xml:space="preserve">Used by Sheets 2 &amp; 3</t>
   </si>
   <si>
+    <t xml:space="preserve">ANNUAL/MONTHLY MIX &amp; OTHER REVENUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual-prepay take rate (% of Launch customers)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40% conservative; SaaS with 17.6% annual discount typically sees 30-50%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI-tool affiliate revenue (£/mo per Launch customer, amortised)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5% take rate × £24/yr commission (Cursor/Anthropic/Lovable/Bolt/Windsurf referrals). Conservative — most customers come AI-tool-first.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual-prepay float yield (£/mo per annual customer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5% APY on £84 avg balance held over the year (half of £168 prepaid).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Per-customer monthly margin — three scenarios</t>
   </si>
   <si>
@@ -250,10 +278,13 @@
     <t xml:space="preserve">Revenue — subscription</t>
   </si>
   <si>
-    <t xml:space="preserve">Revenue — overage markup</t>
+    <t xml:space="preserve">Revenue — overage (pass-through: customer pays cost × (1 + markup))</t>
   </si>
   <si>
     <t xml:space="preserve">Total revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue — other (affiliate + amortised annual-prepay float)</t>
   </si>
   <si>
     <t xml:space="preserve">Less: Paddle fees</t>
@@ -401,17 +432,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\£#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0"/>
-    <numFmt numFmtId="168" formatCode="\£#,##0.00"/>
-    <numFmt numFmtId="169" formatCode="#,##0"/>
-    <numFmt numFmtId="170" formatCode="\£#,##0.00;&quot;(£&quot;#,##0.00\);\-"/>
-    <numFmt numFmtId="171" formatCode="\£#,##0.00;&quot;(£&quot;#,##0.00\);\-"/>
-    <numFmt numFmtId="172" formatCode="0%"/>
-    <numFmt numFmtId="173" formatCode="\£#,##0;&quot;(£&quot;#,##0\);\-"/>
+    <numFmt numFmtId="168" formatCode="#,##0"/>
+    <numFmt numFmtId="169" formatCode="\£#,##0.00;&quot;(£&quot;#,##0.00\);\-"/>
+    <numFmt numFmtId="170" formatCode="0%"/>
+    <numFmt numFmtId="171" formatCode="\£#,##0;&quot;(£&quot;#,##0\);\-"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -611,7 +640,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -652,19 +681,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -673,10 +694,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -700,15 +717,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -732,11 +745,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -748,19 +761,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -768,15 +781,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1059,7 +1072,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="48"/>
@@ -1150,12 +1163,15 @@
         <v>4</v>
       </c>
       <c r="B13" s="7" t="n">
-        <v>14</v>
+        <v>15.8</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B14" s="7" t="n">
         <v>39</v>
@@ -1163,7 +1179,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B15" s="7" t="n">
         <v>89</v>
@@ -1171,7 +1187,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -1180,33 +1196,33 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B18" s="7" t="n">
         <v>3</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B19" s="7" t="n">
         <v>10</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -1215,33 +1231,33 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B22" s="7" t="n">
         <v>1.2</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B23" s="7" t="n">
         <v>7.5</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -1250,46 +1266,46 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B26" s="8" t="n">
         <v>0.3</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B27" s="8" t="n">
         <v>0.6</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B28" s="9" t="n">
         <v>40</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
@@ -1298,46 +1314,44 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B30" s="8" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
+        <v>0.6</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B31" s="7" t="n">
         <v>2</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B32" s="7" t="n">
         <v>5</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -1346,59 +1360,55 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B35" s="7" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
+        <v>2.46</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B36" s="8" t="n">
         <v>0.05</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B37" s="7" t="n">
         <v>0.4</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="B38" s="11" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C38" s="12" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
+      <c r="B38" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
@@ -1407,53 +1417,91 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B40" s="13" t="n">
+        <v>42</v>
+      </c>
+      <c r="B40" s="11" t="n">
         <v>1000</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B41" s="8" t="n">
         <v>0.8</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B43" s="14"/>
-      <c r="C43" s="14"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
+      <c r="A43" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B43" s="12"/>
+      <c r="C43" s="12"/>
+      <c r="D43" s="12"/>
+      <c r="E43" s="12"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B44" s="15" t="n">
+        <v>47</v>
+      </c>
+      <c r="B44" s="13" t="n">
         <f aca="false">cost_cheap*(1-mix_slider/100)+cost_expensive*(mix_slider/100)</f>
         <v>3.72</v>
       </c>
-      <c r="C44" s="16" t="s">
-        <v>47</v>
+      <c r="C44" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B47" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B48" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B49" s="1" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
+  <mergeCells count="24">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A4:E10"/>
@@ -1469,14 +1517,11 @@
     <mergeCell ref="C27:E27"/>
     <mergeCell ref="C28:E28"/>
     <mergeCell ref="A29:E29"/>
-    <mergeCell ref="C30:E30"/>
     <mergeCell ref="C31:E31"/>
     <mergeCell ref="C32:E32"/>
     <mergeCell ref="A34:E34"/>
-    <mergeCell ref="C35:E35"/>
     <mergeCell ref="C36:E36"/>
     <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C38:E38"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="C40:E40"/>
     <mergeCell ref="C41:E41"/>
@@ -1506,7 +1551,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1517,7 +1562,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -1527,29 +1572,29 @@
       <c r="G2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17"/>
-      <c r="B4" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>51</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="E4" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="F4" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>55</v>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -1560,511 +1605,531 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B6" s="18" t="n">
+        <v>65</v>
+      </c>
+      <c r="B6" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="16" t="n">
         <f aca="false">byo_pct</f>
         <v>0.3</v>
       </c>
-      <c r="D6" s="18" t="n">
+      <c r="D6" s="15" t="n">
         <v>0.8</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="16" t="n">
         <f aca="false">byo_pct</f>
         <v>0.3</v>
       </c>
-      <c r="G6" s="18" t="n">
+      <c r="G6" s="15" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" s="18" t="n">
+        <v>66</v>
+      </c>
+      <c r="B7" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="16" t="n">
         <f aca="false">util_pct</f>
         <v>0.6</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="15" t="n">
         <v>0.2</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="16" t="n">
         <f aca="false">util_pct</f>
         <v>0.6</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="G7" s="15" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B8" s="20" t="n">
+        <v>67</v>
+      </c>
+      <c r="B8" s="17" t="n">
         <f aca="false">cost_expensive</f>
         <v>7.5</v>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="17" t="n">
         <f aca="false">cost_blended</f>
         <v>3.72</v>
       </c>
-      <c r="D8" s="20" t="n">
+      <c r="D8" s="17" t="n">
         <f aca="false">cost_cheap</f>
         <v>1.2</v>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E8" s="17" t="n">
         <f aca="false">cost_expensive</f>
         <v>7.5</v>
       </c>
-      <c r="F8" s="20" t="n">
+      <c r="F8" s="17" t="n">
         <f aca="false">cost_blended</f>
         <v>3.72</v>
       </c>
-      <c r="G8" s="20" t="n">
+      <c r="G8" s="17" t="n">
         <f aca="false">cost_cheap</f>
         <v>1.2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B9" s="21" t="n">
-        <f aca="false">overage_launch*1.5</f>
-        <v>3</v>
-      </c>
-      <c r="C9" s="20" t="n">
+        <v>68</v>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="17" t="n">
         <f aca="false">overage_launch</f>
         <v>2</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="18" t="n">
+        <f aca="false">overage_launch</f>
+        <v>2</v>
+      </c>
+      <c r="E9" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="21" t="n">
-        <f aca="false">overage_growth*1.5</f>
-        <v>7.5</v>
-      </c>
-      <c r="F9" s="20" t="n">
+      <c r="F9" s="17" t="n">
         <f aca="false">overage_growth</f>
         <v>5</v>
       </c>
-      <c r="G9" s="21" t="n">
-        <v>0</v>
+      <c r="G9" s="18" t="n">
+        <f aca="false">overage_growth</f>
+        <v>5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
+      <c r="A11" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B12" s="22" t="n">
+        <v>70</v>
+      </c>
+      <c r="B12" s="19" t="n">
         <f aca="false">px_launch_monthly</f>
-        <v>14</v>
-      </c>
-      <c r="C12" s="22" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="C12" s="19" t="n">
         <f aca="false">px_launch_monthly</f>
-        <v>14</v>
-      </c>
-      <c r="D12" s="22" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="D12" s="19" t="n">
         <f aca="false">px_launch_monthly</f>
-        <v>14</v>
-      </c>
-      <c r="E12" s="22" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="E12" s="19" t="n">
         <f aca="false">px_growth_monthly</f>
         <v>39</v>
       </c>
-      <c r="F12" s="22" t="n">
+      <c r="F12" s="19" t="n">
         <f aca="false">px_growth_monthly</f>
         <v>39</v>
       </c>
-      <c r="G12" s="22" t="n">
+      <c r="G12" s="19" t="n">
         <f aca="false">px_growth_monthly</f>
         <v>39</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B13" s="22" t="n">
-        <f aca="false">B9*(1-B6)*overage_markup</f>
-        <v>0.9</v>
-      </c>
-      <c r="C13" s="22" t="n">
-        <f aca="false">C9*(1-C6)*overage_markup</f>
-        <v>0.42</v>
-      </c>
-      <c r="D13" s="22" t="n">
-        <f aca="false">D9*(1-D6)*overage_markup</f>
+        <v>71</v>
+      </c>
+      <c r="B13" s="19" t="n">
+        <f aca="false">B9*(1-B6)*(1+overage_markup)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="22" t="n">
-        <f aca="false">E9*(1-E6)*overage_markup</f>
-        <v>2.25</v>
-      </c>
-      <c r="F13" s="22" t="n">
-        <f aca="false">F9*(1-F6)*overage_markup</f>
-        <v>1.05</v>
-      </c>
-      <c r="G13" s="22" t="n">
-        <f aca="false">G9*(1-G6)*overage_markup</f>
+      <c r="C13" s="19" t="n">
+        <f aca="false">C9*(1-C6)*(1+overage_markup)</f>
+        <v>2.24</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <f aca="false">D9*(1-D6)*(1+overage_markup)</f>
+        <v>0.64</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <f aca="false">E9*(1-E6)*(1+overage_markup)</f>
         <v>0</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <f aca="false">F9*(1-F6)*(1+overage_markup)</f>
+        <v>5.6</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <f aca="false">G9*(1-G6)*(1+overage_markup)</f>
+        <v>1.6</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B14" s="22" t="n">
-        <f aca="false">B12+B13</f>
-        <v>14.9</v>
-      </c>
-      <c r="C14" s="22" t="n">
-        <f aca="false">C12+C13</f>
-        <v>14.42</v>
-      </c>
-      <c r="D14" s="22" t="n">
-        <f aca="false">D12+D13</f>
-        <v>14</v>
-      </c>
-      <c r="E14" s="22" t="n">
-        <f aca="false">E12+E13</f>
-        <v>41.25</v>
-      </c>
-      <c r="F14" s="22" t="n">
-        <f aca="false">F12+F13</f>
-        <v>40.05</v>
-      </c>
-      <c r="G14" s="22" t="n">
-        <f aca="false">G12+G13</f>
-        <v>39</v>
+        <v>72</v>
+      </c>
+      <c r="B14" s="19" t="n">
+        <f aca="false">B12+B13+B15</f>
+        <v>16.04</v>
+      </c>
+      <c r="C14" s="19" t="n">
+        <f aca="false">C12+C13+C15</f>
+        <v>18.28</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <f aca="false">D12+D13+D15</f>
+        <v>16.68</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <f aca="false">E12+E13+E15</f>
+        <v>39.24</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <f aca="false">F12+F13+F15</f>
+        <v>44.84</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <f aca="false">G12+G13+G15</f>
+        <v>40.84</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6"/>
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
+      <c r="A15" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="19" t="n">
+        <f aca="false">affiliate_per_customer+annual_rate*float_per_annual</f>
+        <v>0.24</v>
+      </c>
+      <c r="C15" s="19" t="n">
+        <f aca="false">affiliate_per_customer+annual_rate*float_per_annual</f>
+        <v>0.24</v>
+      </c>
+      <c r="D15" s="19" t="n">
+        <f aca="false">affiliate_per_customer+annual_rate*float_per_annual</f>
+        <v>0.24</v>
+      </c>
+      <c r="E15" s="19" t="n">
+        <f aca="false">affiliate_per_customer+annual_rate*float_per_annual</f>
+        <v>0.24</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <f aca="false">affiliate_per_customer+annual_rate*float_per_annual</f>
+        <v>0.24</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <f aca="false">affiliate_per_customer+annual_rate*float_per_annual</f>
+        <v>0.24</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B16" s="22" t="n">
+        <v>74</v>
+      </c>
+      <c r="B16" s="19" t="n">
         <f aca="false">-(B14*paddle_pct+paddle_fixed)</f>
-        <v>-1.145</v>
-      </c>
-      <c r="C16" s="22" t="n">
+        <v>-1.202</v>
+      </c>
+      <c r="C16" s="19" t="n">
         <f aca="false">-(C14*paddle_pct+paddle_fixed)</f>
-        <v>-1.121</v>
-      </c>
-      <c r="D16" s="22" t="n">
+        <v>-1.314</v>
+      </c>
+      <c r="D16" s="19" t="n">
         <f aca="false">-(D14*paddle_pct+paddle_fixed)</f>
-        <v>-1.1</v>
-      </c>
-      <c r="E16" s="22" t="n">
+        <v>-1.234</v>
+      </c>
+      <c r="E16" s="19" t="n">
         <f aca="false">-(E14*paddle_pct+paddle_fixed)</f>
-        <v>-2.4625</v>
-      </c>
-      <c r="F16" s="22" t="n">
+        <v>-2.362</v>
+      </c>
+      <c r="F16" s="19" t="n">
         <f aca="false">-(F14*paddle_pct+paddle_fixed)</f>
-        <v>-2.4025</v>
-      </c>
-      <c r="G16" s="22" t="n">
+        <v>-2.642</v>
+      </c>
+      <c r="G16" s="19" t="n">
         <f aca="false">-(G14*paddle_pct+paddle_fixed)</f>
-        <v>-2.35</v>
+        <v>-2.442</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B17" s="22" t="n">
+        <v>75</v>
+      </c>
+      <c r="B17" s="19" t="n">
         <f aca="false">-infra_cost</f>
-        <v>-8.5</v>
-      </c>
-      <c r="C17" s="22" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="C17" s="19" t="n">
         <f aca="false">-infra_cost</f>
-        <v>-8.5</v>
-      </c>
-      <c r="D17" s="22" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="D17" s="19" t="n">
         <f aca="false">-infra_cost</f>
-        <v>-8.5</v>
-      </c>
-      <c r="E17" s="22" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="E17" s="19" t="n">
         <f aca="false">-infra_cost</f>
-        <v>-8.5</v>
-      </c>
-      <c r="F17" s="22" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="F17" s="19" t="n">
         <f aca="false">-infra_cost</f>
-        <v>-8.5</v>
-      </c>
-      <c r="G17" s="22" t="n">
+        <v>-2.46</v>
+      </c>
+      <c r="G17" s="19" t="n">
         <f aca="false">-infra_cost</f>
-        <v>-8.5</v>
+        <v>-2.46</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="B18" s="22" t="n">
+        <v>76</v>
+      </c>
+      <c r="B18" s="19" t="n">
         <f aca="false">-allow_launch*B7*(1-B6)</f>
         <v>-3</v>
       </c>
-      <c r="C18" s="22" t="n">
+      <c r="C18" s="19" t="n">
         <f aca="false">-allow_launch*C7*(1-C6)</f>
         <v>-1.26</v>
       </c>
-      <c r="D18" s="22" t="n">
+      <c r="D18" s="19" t="n">
         <f aca="false">-allow_launch*D7*(1-D6)</f>
         <v>-0.12</v>
       </c>
-      <c r="E18" s="22" t="n">
+      <c r="E18" s="19" t="n">
         <f aca="false">-allow_growth*E7*(1-E6)</f>
         <v>-10</v>
       </c>
-      <c r="F18" s="22" t="n">
+      <c r="F18" s="19" t="n">
         <f aca="false">-allow_growth*F7*(1-F6)</f>
         <v>-4.2</v>
       </c>
-      <c r="G18" s="22" t="n">
+      <c r="G18" s="19" t="n">
         <f aca="false">-allow_growth*G7*(1-G6)</f>
         <v>-0.4</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="B19" s="22" t="n">
+        <v>77</v>
+      </c>
+      <c r="B19" s="19" t="n">
         <f aca="false">-B9*(1-B6)</f>
-        <v>-3</v>
-      </c>
-      <c r="C19" s="22" t="n">
+        <v>-0</v>
+      </c>
+      <c r="C19" s="19" t="n">
         <f aca="false">-C9*(1-C6)</f>
         <v>-1.4</v>
       </c>
-      <c r="D19" s="22" t="n">
+      <c r="D19" s="19" t="n">
         <f aca="false">-D9*(1-D6)</f>
+        <v>-0.4</v>
+      </c>
+      <c r="E19" s="19" t="n">
+        <f aca="false">-E9*(1-E6)</f>
         <v>-0</v>
       </c>
-      <c r="E19" s="22" t="n">
-        <f aca="false">-E9*(1-E6)</f>
-        <v>-7.5</v>
-      </c>
-      <c r="F19" s="22" t="n">
+      <c r="F19" s="19" t="n">
         <f aca="false">-F9*(1-F6)</f>
         <v>-3.5</v>
       </c>
-      <c r="G19" s="22" t="n">
+      <c r="G19" s="19" t="n">
         <f aca="false">-G9*(1-G6)</f>
-        <v>-0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="B20" s="23" t="n">
+        <v>78</v>
+      </c>
+      <c r="B20" s="19" t="n">
         <f aca="false">-kept_sandbox_cost</f>
-        <v>-1.5</v>
-      </c>
-      <c r="C20" s="23" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="C20" s="19" t="n">
         <f aca="false">-kept_sandbox_cost</f>
-        <v>-1.5</v>
-      </c>
-      <c r="D20" s="23" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="D20" s="19" t="n">
         <f aca="false">-kept_sandbox_cost</f>
-        <v>-1.5</v>
-      </c>
-      <c r="E20" s="23" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="E20" s="19" t="n">
         <f aca="false">-kept_sandbox_cost</f>
-        <v>-1.5</v>
-      </c>
-      <c r="F20" s="23" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="F20" s="19" t="n">
         <f aca="false">-kept_sandbox_cost</f>
-        <v>-1.5</v>
-      </c>
-      <c r="G20" s="23" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="G20" s="19" t="n">
         <f aca="false">-kept_sandbox_cost</f>
-        <v>-1.5</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B21" s="24" t="n">
+        <v>79</v>
+      </c>
+      <c r="B21" s="20" t="n">
         <f aca="false">SUM(B14,B16:B20)</f>
-        <v>-2.245</v>
-      </c>
-      <c r="C21" s="24" t="n">
+        <v>9.078</v>
+      </c>
+      <c r="C21" s="20" t="n">
         <f aca="false">SUM(C14,C16:C20)</f>
-        <v>0.639</v>
-      </c>
-      <c r="D21" s="24" t="n">
+        <v>11.546</v>
+      </c>
+      <c r="D21" s="20" t="n">
         <f aca="false">SUM(D14,D16:D20)</f>
-        <v>2.78</v>
-      </c>
-      <c r="E21" s="24" t="n">
+        <v>12.166</v>
+      </c>
+      <c r="E21" s="20" t="n">
         <f aca="false">SUM(E14,E16:E20)</f>
-        <v>11.2875</v>
-      </c>
-      <c r="F21" s="24" t="n">
+        <v>24.118</v>
+      </c>
+      <c r="F21" s="20" t="n">
         <f aca="false">SUM(F14,F16:F20)</f>
-        <v>19.9475</v>
-      </c>
-      <c r="G21" s="24" t="n">
+        <v>31.738</v>
+      </c>
+      <c r="G21" s="20" t="n">
         <f aca="false">SUM(G14,G16:G20)</f>
-        <v>26.25</v>
+        <v>34.238</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
+      <c r="A23" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B24" s="22" t="n">
+        <v>81</v>
+      </c>
+      <c r="B24" s="19" t="n">
         <f aca="false">px_setup-5</f>
         <v>84</v>
       </c>
-      <c r="C24" s="22" t="n">
+      <c r="C24" s="19" t="n">
         <f aca="false">px_setup-5</f>
         <v>84</v>
       </c>
-      <c r="D24" s="22" t="n">
+      <c r="D24" s="19" t="n">
         <f aca="false">px_setup-5</f>
         <v>84</v>
       </c>
-      <c r="E24" s="22" t="n">
+      <c r="E24" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="F24" s="22" t="n">
+      <c r="F24" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G24" s="22" t="n">
+      <c r="G24" s="19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="25" t="s">
-        <v>73</v>
-      </c>
-      <c r="B25" s="24" t="n">
+      <c r="A25" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="B25" s="20" t="n">
         <f aca="false">B24+11*B21</f>
-        <v>59.305</v>
-      </c>
-      <c r="C25" s="24" t="n">
+        <v>183.858</v>
+      </c>
+      <c r="C25" s="20" t="n">
         <f aca="false">C24+11*C21</f>
-        <v>91.029</v>
-      </c>
-      <c r="D25" s="24" t="n">
+        <v>211.006</v>
+      </c>
+      <c r="D25" s="20" t="n">
         <f aca="false">D24+11*D21</f>
-        <v>114.58</v>
-      </c>
-      <c r="E25" s="24" t="n">
+        <v>217.826</v>
+      </c>
+      <c r="E25" s="20" t="n">
         <f aca="false">E24+12*E21</f>
-        <v>135.45</v>
-      </c>
-      <c r="F25" s="24" t="n">
+        <v>289.416</v>
+      </c>
+      <c r="F25" s="20" t="n">
         <f aca="false">F24+12*F21</f>
-        <v>239.37</v>
-      </c>
-      <c r="G25" s="24" t="n">
+        <v>380.856</v>
+      </c>
+      <c r="G25" s="20" t="n">
         <f aca="false">G24+12*G21</f>
-        <v>315</v>
+        <v>410.856</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
+      <c r="A27" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B28" s="26" t="n">
+        <v>84</v>
+      </c>
+      <c r="B28" s="22" t="n">
         <f aca="false">C21</f>
-        <v>0.639</v>
-      </c>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
+        <v>11.546</v>
+      </c>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B29" s="27" t="str">
+        <v>85</v>
+      </c>
+      <c r="B29" s="23" t="str">
         <f aca="false">TEXT(B21,"£#,##0.00")&amp;"  →  "&amp;TEXT(D21,"£#,##0.00")</f>
-        <v>-£2.25  →  £2.78</v>
-      </c>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
+        <v>£9.08  →  £12.17</v>
+      </c>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="B30" s="26" t="n">
+        <v>86</v>
+      </c>
+      <c r="B30" s="22" t="n">
         <f aca="false">F21</f>
-        <v>19.9475</v>
-      </c>
-      <c r="C30" s="26"/>
-      <c r="D30" s="26"/>
+        <v>31.738</v>
+      </c>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B31" s="27" t="str">
+        <v>87</v>
+      </c>
+      <c r="B31" s="23" t="str">
         <f aca="false">TEXT(E21,"£#,##0.00")&amp;"  →  "&amp;TEXT(G21,"£#,##0.00")</f>
-        <v>£11.29  →  £26.25</v>
-      </c>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
+        <v>£24.12  →  £34.24</v>
+      </c>
+      <c r="C31" s="23"/>
+      <c r="D31" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -2103,7 +2168,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2115,7 +2180,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2126,468 +2191,468 @@
       <c r="H2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
-        <v>81</v>
-      </c>
-      <c r="B4" s="28"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
+      <c r="A4" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
+      <c r="H4" s="24"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="29" t="s">
-        <v>82</v>
-      </c>
-      <c r="B5" s="30" t="n">
+      <c r="A5" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="30" t="n">
+      <c r="C5" s="26" t="n">
         <v>0.2</v>
       </c>
-      <c r="D5" s="30" t="n">
+      <c r="D5" s="26" t="n">
         <v>0.4</v>
       </c>
-      <c r="E5" s="30" t="n">
+      <c r="E5" s="26" t="n">
         <v>0.6</v>
       </c>
-      <c r="F5" s="30" t="n">
+      <c r="F5" s="26" t="n">
         <v>0.8</v>
       </c>
-      <c r="G5" s="30" t="n">
+      <c r="G5" s="26" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="30" t="n">
+      <c r="A6" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="B6" s="31" t="n">
+      <c r="B6" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A6)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A6)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*B$5*(1-$A6))-(overage_launch*(1-$A6))-kept_sandbox_cost</f>
-        <v>1.47</v>
-      </c>
-      <c r="C6" s="31" t="n">
+        <v>10.99</v>
+      </c>
+      <c r="C6" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A6)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A6)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*C$5*(1-$A6))-(overage_launch*(1-$A6))-kept_sandbox_cost</f>
-        <v>0.869999999999999</v>
-      </c>
-      <c r="D6" s="31" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="D6" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A6)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A6)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*D$5*(1-$A6))-(overage_launch*(1-$A6))-kept_sandbox_cost</f>
-        <v>0.269999999999999</v>
-      </c>
-      <c r="E6" s="31" t="n">
+        <v>9.79</v>
+      </c>
+      <c r="E6" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A6)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A6)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*E$5*(1-$A6))-(overage_launch*(1-$A6))-kept_sandbox_cost</f>
-        <v>-0.330000000000001</v>
-      </c>
-      <c r="F6" s="31" t="n">
+        <v>9.19</v>
+      </c>
+      <c r="F6" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A6)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A6)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*F$5*(1-$A6))-(overage_launch*(1-$A6))-kept_sandbox_cost</f>
-        <v>-0.930000000000002</v>
-      </c>
-      <c r="G6" s="31" t="n">
+        <v>8.59</v>
+      </c>
+      <c r="G6" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A6)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A6)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*G$5*(1-$A6))-(overage_launch*(1-$A6))-kept_sandbox_cost</f>
-        <v>-1.53</v>
+        <v>7.99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="30" t="n">
+      <c r="A7" s="26" t="n">
         <v>0.2</v>
       </c>
-      <c r="B7" s="31" t="n">
+      <c r="B7" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A7)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A7)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*B$5*(1-$A7))-(overage_launch*(1-$A7))-kept_sandbox_cost</f>
-        <v>1.756</v>
-      </c>
-      <c r="C7" s="31" t="n">
+        <v>11.162</v>
+      </c>
+      <c r="C7" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A7)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A7)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*C$5*(1-$A7))-(overage_launch*(1-$A7))-kept_sandbox_cost</f>
-        <v>1.276</v>
-      </c>
-      <c r="D7" s="31" t="n">
+        <v>10.682</v>
+      </c>
+      <c r="D7" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A7)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A7)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*D$5*(1-$A7))-(overage_launch*(1-$A7))-kept_sandbox_cost</f>
-        <v>0.796</v>
-      </c>
-      <c r="E7" s="31" t="n">
+        <v>10.202</v>
+      </c>
+      <c r="E7" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A7)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A7)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*E$5*(1-$A7))-(overage_launch*(1-$A7))-kept_sandbox_cost</f>
-        <v>0.316</v>
-      </c>
-      <c r="F7" s="31" t="n">
+        <v>9.722</v>
+      </c>
+      <c r="F7" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A7)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A7)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*F$5*(1-$A7))-(overage_launch*(1-$A7))-kept_sandbox_cost</f>
-        <v>-0.164000000000001</v>
-      </c>
-      <c r="G7" s="31" t="n">
+        <v>9.242</v>
+      </c>
+      <c r="G7" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A7)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A7)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*G$5*(1-$A7))-(overage_launch*(1-$A7))-kept_sandbox_cost</f>
-        <v>-0.644000000000001</v>
+        <v>8.762</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="30" t="n">
+      <c r="A8" s="26" t="n">
         <v>0.4</v>
       </c>
-      <c r="B8" s="31" t="n">
+      <c r="B8" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A8)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A8)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*B$5*(1-$A8))-(overage_launch*(1-$A8))-kept_sandbox_cost</f>
-        <v>2.042</v>
-      </c>
-      <c r="C8" s="31" t="n">
+        <v>11.334</v>
+      </c>
+      <c r="C8" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A8)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A8)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*C$5*(1-$A8))-(overage_launch*(1-$A8))-kept_sandbox_cost</f>
-        <v>1.682</v>
-      </c>
-      <c r="D8" s="31" t="n">
+        <v>10.974</v>
+      </c>
+      <c r="D8" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A8)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A8)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*D$5*(1-$A8))-(overage_launch*(1-$A8))-kept_sandbox_cost</f>
-        <v>1.322</v>
-      </c>
-      <c r="E8" s="31" t="n">
+        <v>10.614</v>
+      </c>
+      <c r="E8" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A8)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A8)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*E$5*(1-$A8))-(overage_launch*(1-$A8))-kept_sandbox_cost</f>
-        <v>0.961999999999999</v>
-      </c>
-      <c r="F8" s="31" t="n">
+        <v>10.254</v>
+      </c>
+      <c r="F8" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A8)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A8)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*F$5*(1-$A8))-(overage_launch*(1-$A8))-kept_sandbox_cost</f>
-        <v>0.601999999999999</v>
-      </c>
-      <c r="G8" s="31" t="n">
+        <v>9.894</v>
+      </c>
+      <c r="G8" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A8)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A8)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*G$5*(1-$A8))-(overage_launch*(1-$A8))-kept_sandbox_cost</f>
-        <v>0.241999999999999</v>
+        <v>9.534</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="30" t="n">
+      <c r="A9" s="26" t="n">
         <v>0.6</v>
       </c>
-      <c r="B9" s="31" t="n">
+      <c r="B9" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A9)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A9)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*B$5*(1-$A9))-(overage_launch*(1-$A9))-kept_sandbox_cost</f>
-        <v>2.328</v>
-      </c>
-      <c r="C9" s="31" t="n">
+        <v>11.506</v>
+      </c>
+      <c r="C9" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A9)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A9)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*C$5*(1-$A9))-(overage_launch*(1-$A9))-kept_sandbox_cost</f>
-        <v>2.088</v>
-      </c>
-      <c r="D9" s="31" t="n">
+        <v>11.266</v>
+      </c>
+      <c r="D9" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A9)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A9)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*D$5*(1-$A9))-(overage_launch*(1-$A9))-kept_sandbox_cost</f>
-        <v>1.848</v>
-      </c>
-      <c r="E9" s="31" t="n">
+        <v>11.026</v>
+      </c>
+      <c r="E9" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A9)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A9)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*E$5*(1-$A9))-(overage_launch*(1-$A9))-kept_sandbox_cost</f>
-        <v>1.608</v>
-      </c>
-      <c r="F9" s="31" t="n">
+        <v>10.786</v>
+      </c>
+      <c r="F9" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A9)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A9)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*F$5*(1-$A9))-(overage_launch*(1-$A9))-kept_sandbox_cost</f>
-        <v>1.368</v>
-      </c>
-      <c r="G9" s="31" t="n">
+        <v>10.546</v>
+      </c>
+      <c r="G9" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A9)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A9)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*G$5*(1-$A9))-(overage_launch*(1-$A9))-kept_sandbox_cost</f>
-        <v>1.128</v>
+        <v>10.306</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="30" t="n">
+      <c r="A10" s="26" t="n">
         <v>0.8</v>
       </c>
-      <c r="B10" s="31" t="n">
+      <c r="B10" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A10)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A10)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*B$5*(1-$A10))-(overage_launch*(1-$A10))-kept_sandbox_cost</f>
-        <v>2.614</v>
-      </c>
-      <c r="C10" s="31" t="n">
+        <v>11.678</v>
+      </c>
+      <c r="C10" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A10)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A10)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*C$5*(1-$A10))-(overage_launch*(1-$A10))-kept_sandbox_cost</f>
-        <v>2.494</v>
-      </c>
-      <c r="D10" s="31" t="n">
+        <v>11.558</v>
+      </c>
+      <c r="D10" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A10)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A10)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*D$5*(1-$A10))-(overage_launch*(1-$A10))-kept_sandbox_cost</f>
-        <v>2.374</v>
-      </c>
-      <c r="E10" s="31" t="n">
+        <v>11.438</v>
+      </c>
+      <c r="E10" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A10)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A10)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*E$5*(1-$A10))-(overage_launch*(1-$A10))-kept_sandbox_cost</f>
-        <v>2.254</v>
-      </c>
-      <c r="F10" s="31" t="n">
+        <v>11.318</v>
+      </c>
+      <c r="F10" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A10)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A10)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*F$5*(1-$A10))-(overage_launch*(1-$A10))-kept_sandbox_cost</f>
-        <v>2.134</v>
-      </c>
-      <c r="G10" s="31" t="n">
+        <v>11.198</v>
+      </c>
+      <c r="G10" s="27" t="n">
         <f aca="false">px_launch_monthly+(overage_launch*(1-$A10)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A10)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_launch*G$5*(1-$A10))-(overage_launch*(1-$A10))-kept_sandbox_cost</f>
-        <v>2.014</v>
+        <v>11.078</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="28"/>
+      <c r="A12" s="24" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="29" t="s">
-        <v>82</v>
-      </c>
-      <c r="B13" s="30" t="n">
+      <c r="A13" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="B13" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="30" t="n">
+      <c r="C13" s="26" t="n">
         <v>0.2</v>
       </c>
-      <c r="D13" s="30" t="n">
+      <c r="D13" s="26" t="n">
         <v>0.4</v>
       </c>
-      <c r="E13" s="30" t="n">
+      <c r="E13" s="26" t="n">
         <v>0.6</v>
       </c>
-      <c r="F13" s="30" t="n">
+      <c r="F13" s="26" t="n">
         <v>0.8</v>
       </c>
-      <c r="G13" s="30" t="n">
+      <c r="G13" s="26" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="30" t="n">
+      <c r="A14" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="B14" s="31" t="n">
+      <c r="B14" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A14)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A14)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*B$13*(1-$A14))-(overage_growth*(1-$A14))-kept_sandbox_cost</f>
-        <v>23.075</v>
-      </c>
-      <c r="C14" s="31" t="n">
+        <v>31.74</v>
+      </c>
+      <c r="C14" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A14)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A14)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*C$13*(1-$A14))-(overage_growth*(1-$A14))-kept_sandbox_cost</f>
-        <v>21.075</v>
-      </c>
-      <c r="D14" s="31" t="n">
+        <v>29.74</v>
+      </c>
+      <c r="D14" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A14)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A14)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*D$13*(1-$A14))-(overage_growth*(1-$A14))-kept_sandbox_cost</f>
-        <v>19.075</v>
-      </c>
-      <c r="E14" s="31" t="n">
+        <v>27.74</v>
+      </c>
+      <c r="E14" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A14)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A14)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*E$13*(1-$A14))-(overage_growth*(1-$A14))-kept_sandbox_cost</f>
-        <v>17.075</v>
-      </c>
-      <c r="F14" s="31" t="n">
+        <v>25.74</v>
+      </c>
+      <c r="F14" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A14)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A14)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*F$13*(1-$A14))-(overage_growth*(1-$A14))-kept_sandbox_cost</f>
-        <v>15.075</v>
-      </c>
-      <c r="G14" s="31" t="n">
+        <v>23.74</v>
+      </c>
+      <c r="G14" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A14)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A14)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*G$13*(1-$A14))-(overage_growth*(1-$A14))-kept_sandbox_cost</f>
-        <v>13.075</v>
+        <v>21.74</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="30" t="n">
+      <c r="A15" s="26" t="n">
         <v>0.2</v>
       </c>
-      <c r="B15" s="31" t="n">
+      <c r="B15" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A15)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A15)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*B$13*(1-$A15))-(overage_growth*(1-$A15))-kept_sandbox_cost</f>
-        <v>23.79</v>
-      </c>
-      <c r="C15" s="31" t="n">
+        <v>32.17</v>
+      </c>
+      <c r="C15" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A15)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A15)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*C$13*(1-$A15))-(overage_growth*(1-$A15))-kept_sandbox_cost</f>
-        <v>22.19</v>
-      </c>
-      <c r="D15" s="31" t="n">
+        <v>30.57</v>
+      </c>
+      <c r="D15" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A15)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A15)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*D$13*(1-$A15))-(overage_growth*(1-$A15))-kept_sandbox_cost</f>
-        <v>20.59</v>
-      </c>
-      <c r="E15" s="31" t="n">
+        <v>28.97</v>
+      </c>
+      <c r="E15" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A15)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A15)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*E$13*(1-$A15))-(overage_growth*(1-$A15))-kept_sandbox_cost</f>
-        <v>18.99</v>
-      </c>
-      <c r="F15" s="31" t="n">
+        <v>27.37</v>
+      </c>
+      <c r="F15" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A15)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A15)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*F$13*(1-$A15))-(overage_growth*(1-$A15))-kept_sandbox_cost</f>
-        <v>17.39</v>
-      </c>
-      <c r="G15" s="31" t="n">
+        <v>25.77</v>
+      </c>
+      <c r="G15" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A15)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A15)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*G$13*(1-$A15))-(overage_growth*(1-$A15))-kept_sandbox_cost</f>
-        <v>15.79</v>
+        <v>24.17</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="30" t="n">
+      <c r="A16" s="26" t="n">
         <v>0.4</v>
       </c>
-      <c r="B16" s="31" t="n">
+      <c r="B16" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A16)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A16)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*B$13*(1-$A16))-(overage_growth*(1-$A16))-kept_sandbox_cost</f>
-        <v>24.505</v>
-      </c>
-      <c r="C16" s="31" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="C16" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A16)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A16)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*C$13*(1-$A16))-(overage_growth*(1-$A16))-kept_sandbox_cost</f>
-        <v>23.305</v>
-      </c>
-      <c r="D16" s="31" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="D16" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A16)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A16)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*D$13*(1-$A16))-(overage_growth*(1-$A16))-kept_sandbox_cost</f>
-        <v>22.105</v>
-      </c>
-      <c r="E16" s="31" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="E16" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A16)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A16)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*E$13*(1-$A16))-(overage_growth*(1-$A16))-kept_sandbox_cost</f>
-        <v>20.905</v>
-      </c>
-      <c r="F16" s="31" t="n">
+        <v>29</v>
+      </c>
+      <c r="F16" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A16)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A16)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*F$13*(1-$A16))-(overage_growth*(1-$A16))-kept_sandbox_cost</f>
-        <v>19.705</v>
-      </c>
-      <c r="G16" s="31" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="G16" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A16)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A16)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*G$13*(1-$A16))-(overage_growth*(1-$A16))-kept_sandbox_cost</f>
-        <v>18.505</v>
+        <v>26.6</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="30" t="n">
+      <c r="A17" s="26" t="n">
         <v>0.6</v>
       </c>
-      <c r="B17" s="31" t="n">
+      <c r="B17" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A17)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A17)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*B$13*(1-$A17))-(overage_growth*(1-$A17))-kept_sandbox_cost</f>
-        <v>25.22</v>
-      </c>
-      <c r="C17" s="31" t="n">
+        <v>33.03</v>
+      </c>
+      <c r="C17" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A17)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A17)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*C$13*(1-$A17))-(overage_growth*(1-$A17))-kept_sandbox_cost</f>
-        <v>24.42</v>
-      </c>
-      <c r="D17" s="31" t="n">
+        <v>32.23</v>
+      </c>
+      <c r="D17" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A17)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A17)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*D$13*(1-$A17))-(overage_growth*(1-$A17))-kept_sandbox_cost</f>
-        <v>23.62</v>
-      </c>
-      <c r="E17" s="31" t="n">
+        <v>31.43</v>
+      </c>
+      <c r="E17" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A17)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A17)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*E$13*(1-$A17))-(overage_growth*(1-$A17))-kept_sandbox_cost</f>
-        <v>22.82</v>
-      </c>
-      <c r="F17" s="31" t="n">
+        <v>30.63</v>
+      </c>
+      <c r="F17" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A17)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A17)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*F$13*(1-$A17))-(overage_growth*(1-$A17))-kept_sandbox_cost</f>
-        <v>22.02</v>
-      </c>
-      <c r="G17" s="31" t="n">
+        <v>29.83</v>
+      </c>
+      <c r="G17" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A17)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A17)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*G$13*(1-$A17))-(overage_growth*(1-$A17))-kept_sandbox_cost</f>
-        <v>21.22</v>
+        <v>29.03</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="30" t="n">
+      <c r="A18" s="26" t="n">
         <v>0.8</v>
       </c>
-      <c r="B18" s="31" t="n">
+      <c r="B18" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A18)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A18)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*B$13*(1-$A18))-(overage_growth*(1-$A18))-kept_sandbox_cost</f>
-        <v>25.935</v>
-      </c>
-      <c r="C18" s="31" t="n">
+        <v>33.46</v>
+      </c>
+      <c r="C18" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A18)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A18)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*C$13*(1-$A18))-(overage_growth*(1-$A18))-kept_sandbox_cost</f>
-        <v>25.535</v>
-      </c>
-      <c r="D18" s="31" t="n">
+        <v>33.06</v>
+      </c>
+      <c r="D18" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A18)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A18)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*D$13*(1-$A18))-(overage_growth*(1-$A18))-kept_sandbox_cost</f>
-        <v>25.135</v>
-      </c>
-      <c r="E18" s="31" t="n">
+        <v>32.66</v>
+      </c>
+      <c r="E18" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A18)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A18)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*E$13*(1-$A18))-(overage_growth*(1-$A18))-kept_sandbox_cost</f>
-        <v>24.735</v>
-      </c>
-      <c r="F18" s="31" t="n">
+        <v>32.26</v>
+      </c>
+      <c r="F18" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A18)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A18)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*F$13*(1-$A18))-(overage_growth*(1-$A18))-kept_sandbox_cost</f>
-        <v>24.335</v>
-      </c>
-      <c r="G18" s="31" t="n">
+        <v>31.86</v>
+      </c>
+      <c r="G18" s="27" t="n">
         <f aca="false">px_growth_monthly+(overage_growth*(1-$A18)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A18)*overage_markup)*paddle_pct+paddle_fixed)-infra_cost-(allow_growth*G$13*(1-$A18))-(overage_growth*(1-$A18))-kept_sandbox_cost</f>
-        <v>23.935</v>
+        <v>31.46</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
+      <c r="A20" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="29" t="s">
-        <v>85</v>
-      </c>
-      <c r="B21" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="C21" s="29" t="s">
-        <v>87</v>
+      <c r="A21" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="30" t="n">
+      <c r="A22" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="B22" s="32" t="n">
+      <c r="B22" s="28" t="n">
         <f aca="false">IFERROR(IF((allow_launch*(1-$A22))=0,"n/a (BYO=100%)",MAX(0,((px_launch_monthly+overage_launch*(1-$A22)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A22)*overage_markup)*paddle_pct+paddle_fixed+infra_cost+kept_sandbox_cost+overage_launch*(1-$A22)))/(allow_launch*(1-$A22)))),"err")</f>
-        <v>0.49</v>
-      </c>
-      <c r="C22" s="32" t="n">
+        <v>3.66333333333333</v>
+      </c>
+      <c r="C22" s="28" t="n">
         <f aca="false">IFERROR(IF((allow_growth*(1-$A22))=0,"n/a (BYO=100%)",MAX(0,((px_growth_monthly+overage_growth*(1-$A22)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A22)*overage_markup)*paddle_pct+paddle_fixed+infra_cost+kept_sandbox_cost+overage_growth*(1-$A22)))/(allow_growth*(1-$A22)))),"err")</f>
-        <v>2.3075</v>
+        <v>3.174</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="30" t="n">
+      <c r="A23" s="26" t="n">
         <v>0.2</v>
       </c>
-      <c r="B23" s="32" t="n">
+      <c r="B23" s="28" t="n">
         <f aca="false">IFERROR(IF((allow_launch*(1-$A23))=0,"n/a (BYO=100%)",MAX(0,((px_launch_monthly+overage_launch*(1-$A23)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A23)*overage_markup)*paddle_pct+paddle_fixed+infra_cost+kept_sandbox_cost+overage_launch*(1-$A23)))/(allow_launch*(1-$A23)))),"err")</f>
-        <v>0.731666666666667</v>
-      </c>
-      <c r="C23" s="32" t="n">
+        <v>4.65083333333333</v>
+      </c>
+      <c r="C23" s="28" t="n">
         <f aca="false">IFERROR(IF((allow_growth*(1-$A23))=0,"n/a (BYO=100%)",MAX(0,((px_growth_monthly+overage_growth*(1-$A23)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A23)*overage_markup)*paddle_pct+paddle_fixed+infra_cost+kept_sandbox_cost+overage_growth*(1-$A23)))/(allow_growth*(1-$A23)))),"err")</f>
-        <v>2.97375</v>
+        <v>4.02125</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="30" t="n">
+      <c r="A24" s="26" t="n">
         <v>0.4</v>
       </c>
-      <c r="B24" s="32" t="n">
+      <c r="B24" s="28" t="n">
         <f aca="false">IFERROR(IF((allow_launch*(1-$A24))=0,"n/a (BYO=100%)",MAX(0,((px_launch_monthly+overage_launch*(1-$A24)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A24)*overage_markup)*paddle_pct+paddle_fixed+infra_cost+kept_sandbox_cost+overage_launch*(1-$A24)))/(allow_launch*(1-$A24)))),"err")</f>
-        <v>1.13444444444444</v>
-      </c>
-      <c r="C24" s="32" t="n">
+        <v>6.29666666666667</v>
+      </c>
+      <c r="C24" s="28" t="n">
         <f aca="false">IFERROR(IF((allow_growth*(1-$A24))=0,"n/a (BYO=100%)",MAX(0,((px_growth_monthly+overage_growth*(1-$A24)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A24)*overage_markup)*paddle_pct+paddle_fixed+infra_cost+kept_sandbox_cost+overage_growth*(1-$A24)))/(allow_growth*(1-$A24)))),"err")</f>
-        <v>4.08416666666667</v>
+        <v>5.43333333333333</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="30" t="n">
+      <c r="A25" s="26" t="n">
         <v>0.6</v>
       </c>
-      <c r="B25" s="32" t="n">
+      <c r="B25" s="28" t="n">
         <f aca="false">IFERROR(IF((allow_launch*(1-$A25))=0,"n/a (BYO=100%)",MAX(0,((px_launch_monthly+overage_launch*(1-$A25)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A25)*overage_markup)*paddle_pct+paddle_fixed+infra_cost+kept_sandbox_cost+overage_launch*(1-$A25)))/(allow_launch*(1-$A25)))),"err")</f>
-        <v>1.94</v>
-      </c>
-      <c r="C25" s="32" t="n">
+        <v>9.58833333333333</v>
+      </c>
+      <c r="C25" s="28" t="n">
         <f aca="false">IFERROR(IF((allow_growth*(1-$A25))=0,"n/a (BYO=100%)",MAX(0,((px_growth_monthly+overage_growth*(1-$A25)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A25)*overage_markup)*paddle_pct+paddle_fixed+infra_cost+kept_sandbox_cost+overage_growth*(1-$A25)))/(allow_growth*(1-$A25)))),"err")</f>
-        <v>6.305</v>
+        <v>8.2575</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="30" t="n">
+      <c r="A26" s="26" t="n">
         <v>0.8</v>
       </c>
-      <c r="B26" s="32" t="n">
+      <c r="B26" s="28" t="n">
         <f aca="false">IFERROR(IF((allow_launch*(1-$A26))=0,"n/a (BYO=100%)",MAX(0,((px_launch_monthly+overage_launch*(1-$A26)*overage_markup)-((px_launch_monthly+overage_launch*(1-$A26)*overage_markup)*paddle_pct+paddle_fixed+infra_cost+kept_sandbox_cost+overage_launch*(1-$A26)))/(allow_launch*(1-$A26)))),"err")</f>
-        <v>4.35666666666667</v>
-      </c>
-      <c r="C26" s="32" t="n">
+        <v>19.4633333333333</v>
+      </c>
+      <c r="C26" s="28" t="n">
         <f aca="false">IFERROR(IF((allow_growth*(1-$A26))=0,"n/a (BYO=100%)",MAX(0,((px_growth_monthly+overage_growth*(1-$A26)*overage_markup)-((px_growth_monthly+overage_growth*(1-$A26)*overage_markup)*paddle_pct+paddle_fixed+infra_cost+kept_sandbox_cost+overage_growth*(1-$A26)))/(allow_growth*(1-$A26)))),"err")</f>
-        <v>12.9675</v>
+        <v>16.73</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="33" t="s">
-        <v>88</v>
-      </c>
-      <c r="B28" s="33"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
+      <c r="A28" s="29" t="s">
+        <v>97</v>
+      </c>
+      <c r="B28" s="29"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="33"/>
-      <c r="B29" s="33"/>
-      <c r="C29" s="33"/>
-      <c r="D29" s="33"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="33"/>
+      <c r="A29" s="29"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="29"/>
+      <c r="F29" s="29"/>
+      <c r="G29" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2646,7 +2711,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2655,7 +2720,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2663,215 +2728,215 @@
       <c r="E2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
+      <c r="A4" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="B5" s="34" t="n">
+        <v>101</v>
+      </c>
+      <c r="B5" s="30" t="n">
         <f aca="false">cohort_total</f>
         <v>1000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B6" s="19" t="n">
+        <v>102</v>
+      </c>
+      <c r="B6" s="16" t="n">
         <f aca="false">cohort_launch_pct</f>
         <v>0.8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B7" s="19" t="n">
+        <v>103</v>
+      </c>
+      <c r="B7" s="16" t="n">
         <f aca="false">1-cohort_launch_pct</f>
         <v>0.2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="B8" s="34" t="n">
+        <v>104</v>
+      </c>
+      <c r="B8" s="30" t="n">
         <f aca="false">B5*B6</f>
         <v>800</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="B9" s="34" t="n">
+        <v>105</v>
+      </c>
+      <c r="B9" s="30" t="n">
         <f aca="false">B5*B7</f>
         <v>200</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
+      <c r="A11" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17"/>
-      <c r="B12" s="17" t="s">
-        <v>98</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>99</v>
-      </c>
-      <c r="D12" s="17" t="s">
-        <v>100</v>
+      <c r="A12" s="14"/>
+      <c r="B12" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="B13" s="35" t="n">
+        <v>110</v>
+      </c>
+      <c r="B13" s="31" t="n">
         <f aca="false">px_setup+11*(px_launch_monthly+'Per-customer margin'!C13)</f>
-        <v>247.62</v>
-      </c>
-      <c r="C13" s="35" t="n">
+        <v>287.44</v>
+      </c>
+      <c r="C13" s="31" t="n">
         <f aca="false">12*(px_growth_monthly+'Per-customer margin'!F13)</f>
-        <v>480.6</v>
-      </c>
-      <c r="D13" s="35" t="n">
+        <v>535.2</v>
+      </c>
+      <c r="D13" s="31" t="n">
         <f aca="false">B13*B8+C13*B9</f>
-        <v>294216</v>
+        <v>336992</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="B14" s="36" t="n">
+        <v>111</v>
+      </c>
+      <c r="B14" s="32" t="n">
         <f aca="false">year1_launch_mid</f>
-        <v>91.029</v>
-      </c>
-      <c r="C14" s="36" t="n">
+        <v>211.006</v>
+      </c>
+      <c r="C14" s="32" t="n">
         <f aca="false">year1_growth_mid</f>
-        <v>239.37</v>
-      </c>
-      <c r="D14" s="35" t="n">
+        <v>380.856</v>
+      </c>
+      <c r="D14" s="31" t="n">
         <f aca="false">B14*B8+C14*B9</f>
-        <v>120697.2</v>
+        <v>244976</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B15" s="35" t="n">
+        <v>112</v>
+      </c>
+      <c r="B15" s="31" t="n">
         <f aca="false">B13*B8</f>
-        <v>198096</v>
-      </c>
-      <c r="C15" s="35" t="n">
+        <v>229952</v>
+      </c>
+      <c r="C15" s="31" t="n">
         <f aca="false">C13*B9</f>
-        <v>96120</v>
-      </c>
-      <c r="D15" s="37" t="n">
+        <v>107040</v>
+      </c>
+      <c r="D15" s="33" t="n">
         <f aca="false">B15+C15</f>
-        <v>294216</v>
+        <v>336992</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="B16" s="35" t="n">
+        <v>113</v>
+      </c>
+      <c r="B16" s="31" t="n">
         <f aca="false">B14*B8</f>
-        <v>72823.2</v>
-      </c>
-      <c r="C16" s="35" t="n">
+        <v>168804.8</v>
+      </c>
+      <c r="C16" s="31" t="n">
         <f aca="false">C14*B9</f>
-        <v>47874</v>
-      </c>
-      <c r="D16" s="37" t="n">
+        <v>76171.2</v>
+      </c>
+      <c r="D16" s="33" t="n">
         <f aca="false">B16+C16</f>
-        <v>120697.2</v>
+        <v>244976</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B17" s="38" t="n">
+        <v>114</v>
+      </c>
+      <c r="B17" s="34" t="n">
         <f aca="false">B16/B15</f>
-        <v>0.367615701478071</v>
-      </c>
-      <c r="C17" s="38" t="n">
+        <v>0.734087113832452</v>
+      </c>
+      <c r="C17" s="34" t="n">
         <f aca="false">C16/C15</f>
-        <v>0.498064918851436</v>
-      </c>
-      <c r="D17" s="38" t="n">
+        <v>0.711614349775785</v>
+      </c>
+      <c r="D17" s="34" t="n">
         <f aca="false">D16/D15</f>
-        <v>0.410233297985154</v>
+        <v>0.726949007691577</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
+      <c r="A19" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="B20" s="39" t="n">
+        <v>116</v>
+      </c>
+      <c r="B20" s="35" t="n">
         <v>108</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B21" s="39" t="n">
+        <v>117</v>
+      </c>
+      <c r="B21" s="35" t="n">
         <v>338</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="B22" s="40" t="n">
+        <v>118</v>
+      </c>
+      <c r="B22" s="36" t="n">
         <f aca="false">B20*B8+B21*B9</f>
         <v>154000</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B23" s="41" t="n">
+        <v>119</v>
+      </c>
+      <c r="B23" s="37" t="n">
         <f aca="false">D16-B22</f>
-        <v>-33302.8</v>
+        <v>90976</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="B24" s="42" t="n">
+        <v>120</v>
+      </c>
+      <c r="B24" s="38" t="n">
         <f aca="false">B23/B22</f>
-        <v>-0.216251948051948</v>
+        <v>0.590753246753247</v>
       </c>
     </row>
   </sheetData>

</xml_diff>